<commit_message>
Show score and result in the route sheet
Fill optional "Оценка" and "Результат" columns in the route-sheet
template so the user can see each point's indicators and why it was
ordered earlier. Sample data updated to include both columns.
</commit_message>
<xml_diff>
--- a/sample_data/planning.xlsx
+++ b/sample_data/planning.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,16 @@
           <t>Цикличность</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Оценка</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Результат</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -575,6 +585,12 @@
       <c r="Q2" t="n">
         <v>1</v>
       </c>
+      <c r="R2" t="n">
+        <v>5</v>
+      </c>
+      <c r="S2" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -648,6 +664,12 @@
       <c r="Q3" t="n">
         <v>2</v>
       </c>
+      <c r="R3" t="n">
+        <v>4</v>
+      </c>
+      <c r="S3" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -725,6 +747,12 @@
       <c r="Q4" t="n">
         <v>3</v>
       </c>
+      <c r="R4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -798,6 +826,10 @@
       <c r="Q5" t="n">
         <v>4</v>
       </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -879,6 +911,12 @@
       <c r="Q6" t="n">
         <v>1</v>
       </c>
+      <c r="R6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -951,6 +989,12 @@
       </c>
       <c r="Q7" t="n">
         <v>2</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -1021,6 +1065,10 @@
       <c r="Q8" t="n">
         <v>1</v>
       </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1090,6 +1138,12 @@
       <c r="Q9" t="n">
         <v>1</v>
       </c>
+      <c r="R9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1159,6 +1213,12 @@
       <c r="Q10" t="n">
         <v>2</v>
       </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1228,6 +1288,12 @@
       <c r="Q11" t="n">
         <v>3</v>
       </c>
+      <c r="R11" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>150</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Show result as percentage in the route sheet
Result values are percentages, so the exporter now appends "%" when the
base stores a plain number (80 -> "80%"), while preserving an existing
percent sign. Sample data updated to 0-100 percentage values.
</commit_message>
<xml_diff>
--- a/sample_data/planning.xlsx
+++ b/sample_data/planning.xlsx
@@ -589,7 +589,7 @@
         <v>5</v>
       </c>
       <c r="S2" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
@@ -668,7 +668,7 @@
         <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -915,7 +915,7 @@
         <v>3</v>
       </c>
       <c r="S6" t="n">
-        <v>200</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7">
@@ -1292,7 +1292,7 @@
         <v>5</v>
       </c>
       <c r="S11" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>